<commit_message>
Belamcanda: name the plant and add its picture (1.0.1)
"בלה מקנדה" is Belamcanda chinensis (blackberry lily): iris-like sword leaves
and thin branching stems with small orange flowers. It gets its Russian and
English names (no longer "(?)"), a description in data/photo-prompts.xlsx and
a generated picture; 177 of 180 items now have one.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/photo-prompts.xlsx
+++ b/data/photo-prompts.xlsx
@@ -3164,27 +3164,27 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="4" t="n">
+      <c r="A109" s="2" t="n">
         <v>112</v>
       </c>
-      <c r="B109" s="5" t="inlineStr">
+      <c r="B109" s="3" t="inlineStr">
         <is>
           <t>בלה מקנדה</t>
         </is>
       </c>
-      <c r="C109" s="4" t="inlineStr">
-        <is>
-          <t>bella-of-canada</t>
-        </is>
-      </c>
-      <c r="D109" s="4" t="inlineStr">
-        <is>
-          <t>a bunch of thin wiry stems with tiny pale pink buds at the tips and narrow grass-like leaves at the base</t>
-        </is>
-      </c>
-      <c r="E109" s="6" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>belamcanda</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>a few stems of Belamcanda chinensis (blackberry lily): a fan of flat sword-shaped iris-like green leaves at the base and tall thin branching stems with small orange star-shaped flowers and buds at the tips</t>
+        </is>
+      </c>
+      <c r="E109" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
More realistic flower pictures, as chosen by the florist (1.0.3)
32 flower pictures are replaced by new ones generated with a "real cut stem
as sold at a flower market" prompt (fewer flowers per stem, buds, natural
asymmetry): asclepias, alstroemeria, lilies, lisianthus in one colour,
celosias, chrysanthemums, phlox, snapdragon, tweedia blue and more. For the
single-headed flowers (roses, gerberas, callas, anthuriums, orchids, tulip…)
she kept the earlier pictures. Five more (callicarpa, balloon plant, red
hibiscus, limonium, white tweedia) have new descriptions and will be redone.

The prompt no longer asks for leaves by default, so leafless stems can be
described as such.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/photo-prompts.xlsx
+++ b/data/photo-prompts.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>single stem of alstroemeria with a cluster of open pink and white freckled flowers</t>
+          <t>a single cut stem of alstroemeria with a few open pink freckled flowers and some buds on short branching flower stalks, narrow twisted leaves</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>single stem of Asclepias tuberosa (butterfly weed) with a flat cluster of bright orange flowers</t>
+          <t>a single cut stem of Asclepias tuberosa (butterfly weed) with three or four small loose umbels of orange flowers at slightly different heights, some umbels still in yellow-green bud, and many narrow lance-shaped leaves along the stem</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>a single branch of red-leaved hibiscus (Hibiscus acetosella) with burgundy maple-like leaves</t>
+          <t>a single bare reddish-purple woody stem of red hibiscus (Hibiscus sabdariffa, roselle) with all leaves removed, carrying fleshy pointed deep-red calyx buds spaced along the upper part of the stem; no leaves, no open flowers</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>single stem of Tweedia caerulea with small star-shaped white flowers and soft grey-green leaves</t>
+          <t>single stem of Tweedia caerulea with small star-shaped pure white flowers and soft grey-green leaves</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>single stem of lisianthus (eustoma) with several ruffled white and purple flowers and buds</t>
+          <t>a single cut stem of lisianthus (eustoma) in one colour, purple, with two open ruffled flowers and several closed buds</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>single stem of Asiatic lily with several open orange flowers and buds</t>
+          <t>a single cut stem of Asiatic lily with two or three open orange flowers and a few closed buds</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>single stem of lily 'Sweet Sugar' with several open soft pink flowers</t>
+          <t>a single cut stem of lily 'Sweet Sugar' with two open soft pink flowers and a couple of closed buds</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>a single branch of Limonium 'Emille' (statice) with clouds of tiny lavender-purple flowers</t>
+          <t>a single cut stem of Limonium 'Emille' (statice): one very thin, wiry, rigid green stem that branches into many fine airy side branches, each tipped with small one-sided sprays of tiny lavender-purple papery flowers; delicate and airy with lots of white space between the branches; no large leaves</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>a single branch of Gomphocarpus physocarpus 'Moby Dick' with round pale green spiky balloon pods and narrow leaves</t>
+          <t>a single cut stem of Gomphocarpus physocarpus (balloon plant) with three to five inflated, slightly pointed, translucent pale lime-green balloon-shaped seed pods covered in soft bristles, hanging on short stalks at different heights, and a few narrow lance-shaped pale green leaves along the stem</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>a single branch of Callicarpa (beautyberry) with clusters of glossy violet berries</t>
+          <t>a single bare woody branch of Callicarpa (beautyberry) as florists sell it, with all leaves stripped off: tight round clusters of small glossy violet-purple berries encircling the stem at intervals along its length, and nothing else on the stem; no leaves</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>single stem of oriental lily with several large open white flowers and buds</t>
+          <t>a single cut stem of oriental lily with two or three large open white flowers and a few closed buds</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>single stem of double oriental lily with several large many-petalled white flowers</t>
+          <t>a single cut stem of double oriental lily with two large many-petalled white flowers and a few closed buds</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>single stem of oriental lily with several large open pale yellow flowers</t>
+          <t>a single cut stem of oriental lily with two open pale yellow flowers and a few closed buds</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>single stem of double oriental lily with several large many-petalled pink flowers</t>
+          <t>a single cut stem of double oriental lily with two large many-petalled pink flowers and a few closed buds</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>single stem of Easter lily (Lilium longiflorum) with white trumpet flowers and green buds</t>
+          <t>a single cut stem of Easter lily (Lilium longiflorum) with one or two white trumpet flowers and green buds</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>single stem of Easter lily (Lilium longiflorum) with white trumpet flowers and green buds</t>
+          <t>a single cut stem of Easter lily (Lilium longiflorum) with one or two white trumpet flowers and green buds</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>single stem of Easter lily (Lilium longiflorum) with white trumpet flowers and green buds</t>
+          <t>a single cut stem of Easter lily (Lilium longiflorum) with one or two white trumpet flowers and green buds</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>single stem of lily with fully open white flowers, stamens removed</t>
+          <t>a single cut stem of lily with two or three fully open white flowers, stamens removed</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">

</xml_diff>